<commit_message>
Changes of sep 2nd
</commit_message>
<xml_diff>
--- a/SeleniumBDDFramework/SeleniumBDDFramework/src/test/resources/TestData/CRMActivityData.xlsx
+++ b/SeleniumBDDFramework/SeleniumBDDFramework/src/test/resources/TestData/CRMActivityData.xlsx
@@ -13,6 +13,7 @@
   <sheets>
     <sheet name="General Activity" sheetId="1" r:id="rId1"/>
     <sheet name="Linked Activity" sheetId="2" r:id="rId2"/>
+    <sheet name="Leads" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr/>
 </workbook>
@@ -201,7 +202,7 @@
     <t>Automated Linked activity</t>
   </si>
   <si>
-    <t>Delhi Public School</t>
+    <t>Sahithi Vidhyalayam High school</t>
   </si>
   <si>
     <t>interview</t>
@@ -210,7 +211,7 @@
     <t>Opportunity</t>
   </si>
   <si>
-    <t>Aarav Sharma</t>
+    <t>Divya sharma</t>
   </si>
   <si>
     <t>Oakridge International School</t>
@@ -1288,7 +1289,7 @@
   <cols>
     <col min="1" max="1" width="26.59766" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="16.29688" customWidth="1"/>
+    <col min="3" max="3" width="26.89844" customWidth="1"/>
     <col min="4" max="4" width="18.09766" customWidth="1"/>
     <col min="5" max="5" width="12.79688" customWidth="1"/>
     <col min="6" max="6" width="48" customWidth="1"/>
@@ -1874,4 +1875,11 @@
     </row>
   </sheetData>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="13.8"/>
+  <sheetData/>
+</worksheet>
 </file>
</xml_diff>